<commit_message>
Add M02 company name change and register templates
</commit_message>
<xml_diff>
--- a/templates/import/P1_registration_sample_v3_1.xlsx
+++ b/templates/import/P1_registration_sample_v3_1.xlsx
@@ -358,6 +358,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
@@ -621,12 +622,12 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>上传后检查董事、秘书、股东股份合计、RORC 控制人、Form 24 和股权证书签字逻辑。</t>
+          <t>上传后检查董事、秘书、股东股份合计、RORC 控制人、M06 registers、Form 24 和股权证书签字逻辑。</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>Review directors, secretary, share totals, RORC, Form 24 and certificate signing.</t>
+          <t>Review directors, secretary, share totals, RORC, M06 registers, Form 24 and certificate signing.</t>
         </is>
       </c>
     </row>
@@ -678,7 +679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23.75" customWidth="1" min="1" max="1"/>
@@ -1472,62 +1473,146 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>任务类型</t>
+          <t>挂名董事提名人姓名覆盖</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Task type</t>
+          <t>Nominee director nominator name override</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
         <is>
-          <t>task_type</t>
-        </is>
-      </c>
-      <c r="D29" s="15" t="inlineStr">
-        <is>
-          <t>incorporation</t>
-        </is>
-      </c>
+          <t>nominee_director_nominator_name</t>
+        </is>
+      </c>
+      <c r="D29" s="15" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Optional</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>固定值，不要修改。</t>
+          <t>通常留空；系统默认第一个客户董事。特殊情况才填写。</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>挂名董事提名人证件号覆盖</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Nominee director nominator ID override</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="inlineStr">
+        <is>
+          <t>nominee_director_nominator_id_number</t>
+        </is>
+      </c>
+      <c r="D30" s="15" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
+        <is>
+          <t>通常留空；与上方姓名一起用于 M06 register。</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>挂名董事提名人地址覆盖</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Nominee director nominator address override</t>
+        </is>
+      </c>
+      <c r="C31" s="12" t="inlineStr">
+        <is>
+          <t>nominee_director_nominator_address</t>
+        </is>
+      </c>
+      <c r="D31" s="15" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="F31" s="9" t="inlineStr">
+        <is>
+          <t>通常留空；与上方姓名一起用于 M06 register。</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>任务类型</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Task type</t>
+        </is>
+      </c>
+      <c r="C32" s="12" t="inlineStr">
+        <is>
+          <t>task_type</t>
+        </is>
+      </c>
+      <c r="D32" s="15" t="inlineStr">
+        <is>
+          <t>incorporation</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="F32" s="9" t="inlineStr">
+        <is>
+          <t>固定值，不要修改。</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
           <t>内部备注</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>Internal remarks</t>
         </is>
       </c>
-      <c r="C30" s="12" t="inlineStr">
+      <c r="C33" s="12" t="inlineStr">
         <is>
           <t>remarks</t>
         </is>
       </c>
-      <c r="D30" s="15" t="inlineStr">
+      <c r="D33" s="15" t="inlineStr">
         <is>
           <t>Sample: issued share capital and paid-up share capital are filled at shareholder level.</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E33" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="F30" s="9" t="inlineStr">
+      <c r="F33" s="9" t="inlineStr">
         <is>
           <t>不进入正式文件。</t>
         </is>
@@ -1573,7 +1658,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
@@ -2448,7 +2532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N19"/>
+  <dimension ref="A1:N26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.5" customWidth="1" min="1" max="1"/>
@@ -3070,30 +3154,26 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>备注</t>
+          <t>是否登记控制人覆盖</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Remarks</t>
+          <t>Registrable controller override</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>remarks</t>
-        </is>
-      </c>
-      <c r="D19" s="9" t="str"/>
-      <c r="E19" s="15" t="inlineStr">
-        <is>
-          <t>70% shareholder.</t>
-        </is>
-      </c>
-      <c r="F19" s="15" t="inlineStr">
-        <is>
-          <t>30% shareholder.</t>
-        </is>
-      </c>
+          <t>is_registrable_controller</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>通常留空=Auto；系统按 25% 股权规则判断。特殊情况可填 Yes/No。</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr"/>
+      <c r="F19" s="15" t="inlineStr"/>
       <c r="G19" s="15" t="inlineStr"/>
       <c r="H19" s="15" t="inlineStr"/>
       <c r="I19" s="15" t="inlineStr"/>
@@ -3103,13 +3183,253 @@
       <c r="M19" s="15" t="inlineStr"/>
       <c r="N19" s="15" t="inlineStr"/>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>控制人依据覆盖</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Controller basis override</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>controller_basis</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>通常留空；特殊控制权安排才填写。</t>
+        </is>
+      </c>
+      <c r="E20" s="15" t="inlineStr"/>
+      <c r="F20" s="15" t="inlineStr"/>
+      <c r="G20" s="15" t="inlineStr"/>
+      <c r="H20" s="15" t="inlineStr"/>
+      <c r="I20" s="15" t="inlineStr"/>
+      <c r="J20" s="15" t="inlineStr"/>
+      <c r="K20" s="15" t="inlineStr"/>
+      <c r="L20" s="15" t="inlineStr"/>
+      <c r="M20" s="15" t="inlineStr"/>
+      <c r="N20" s="15" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>控制人登记日期</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Controller entry date</t>
+        </is>
+      </c>
+      <c r="C21" s="12" t="inlineStr">
+        <is>
+          <t>controller_start_date</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>通常留空=注册日期。</t>
+        </is>
+      </c>
+      <c r="E21" s="15" t="inlineStr"/>
+      <c r="F21" s="15" t="inlineStr"/>
+      <c r="G21" s="15" t="inlineStr"/>
+      <c r="H21" s="15" t="inlineStr"/>
+      <c r="I21" s="15" t="inlineStr"/>
+      <c r="J21" s="15" t="inlineStr"/>
+      <c r="K21" s="15" t="inlineStr"/>
+      <c r="L21" s="15" t="inlineStr"/>
+      <c r="M21" s="15" t="inlineStr"/>
+      <c r="N21" s="15" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>是否挂名股东</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Nominee shareholder</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>is_nominee_shareholder</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>通常留空=No；只有 nominee shareholder 情况填 Yes。</t>
+        </is>
+      </c>
+      <c r="E22" s="15" t="inlineStr"/>
+      <c r="F22" s="15" t="inlineStr"/>
+      <c r="G22" s="15" t="inlineStr"/>
+      <c r="H22" s="15" t="inlineStr"/>
+      <c r="I22" s="15" t="inlineStr"/>
+      <c r="J22" s="15" t="inlineStr"/>
+      <c r="K22" s="15" t="inlineStr"/>
+      <c r="L22" s="15" t="inlineStr"/>
+      <c r="M22" s="15" t="inlineStr"/>
+      <c r="N22" s="15" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>挂名股东提名人/受益人</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Nominee shareholder nominator / beneficial owner</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>nominee_shareholder_nominator_name</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>通常留空；只有挂名股东情况填写。</t>
+        </is>
+      </c>
+      <c r="E23" s="15" t="inlineStr"/>
+      <c r="F23" s="15" t="inlineStr"/>
+      <c r="G23" s="15" t="inlineStr"/>
+      <c r="H23" s="15" t="inlineStr"/>
+      <c r="I23" s="15" t="inlineStr"/>
+      <c r="J23" s="15" t="inlineStr"/>
+      <c r="K23" s="15" t="inlineStr"/>
+      <c r="L23" s="15" t="inlineStr"/>
+      <c r="M23" s="15" t="inlineStr"/>
+      <c r="N23" s="15" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>挂名股东提名人证件号</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Nominee shareholder nominator ID</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="inlineStr">
+        <is>
+          <t>nominee_shareholder_nominator_id_number</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>通常留空。</t>
+        </is>
+      </c>
+      <c r="E24" s="15" t="inlineStr"/>
+      <c r="F24" s="15" t="inlineStr"/>
+      <c r="G24" s="15" t="inlineStr"/>
+      <c r="H24" s="15" t="inlineStr"/>
+      <c r="I24" s="15" t="inlineStr"/>
+      <c r="J24" s="15" t="inlineStr"/>
+      <c r="K24" s="15" t="inlineStr"/>
+      <c r="L24" s="15" t="inlineStr"/>
+      <c r="M24" s="15" t="inlineStr"/>
+      <c r="N24" s="15" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>挂名股东提名人地址</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Nominee shareholder nominator address</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>nominee_shareholder_nominator_address</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>通常留空。</t>
+        </is>
+      </c>
+      <c r="E25" s="15" t="inlineStr"/>
+      <c r="F25" s="15" t="inlineStr"/>
+      <c r="G25" s="15" t="inlineStr"/>
+      <c r="H25" s="15" t="inlineStr"/>
+      <c r="I25" s="15" t="inlineStr"/>
+      <c r="J25" s="15" t="inlineStr"/>
+      <c r="K25" s="15" t="inlineStr"/>
+      <c r="L25" s="15" t="inlineStr"/>
+      <c r="M25" s="15" t="inlineStr"/>
+      <c r="N25" s="15" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="inlineStr">
+        <is>
+          <t>remarks</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="str"/>
+      <c r="E26" s="15" t="inlineStr">
+        <is>
+          <t>70% shareholder.</t>
+        </is>
+      </c>
+      <c r="F26" s="15" t="inlineStr">
+        <is>
+          <t>30% shareholder.</t>
+        </is>
+      </c>
+      <c r="G26" s="15" t="inlineStr"/>
+      <c r="H26" s="15" t="inlineStr"/>
+      <c r="I26" s="15" t="inlineStr"/>
+      <c r="J26" s="15" t="inlineStr"/>
+      <c r="K26" s="15" t="inlineStr"/>
+      <c r="L26" s="15" t="inlineStr"/>
+      <c r="M26" s="15" t="inlineStr"/>
+      <c r="N26" s="15" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
-  <dataValidations count="1">
+  <dataValidations count="5">
     <dataValidation sqref="E4:N4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"person,corporate"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E19:N19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Auto,Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E22:N22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Auto,Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E19:N19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Auto,Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E22:N22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Auto,Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3140,7 +3460,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>

</xml_diff>